<commit_message>
ejercicio 10 y 11
</commit_message>
<xml_diff>
--- a/ejercicios/ej10/data/inventario_limpio.xlsx
+++ b/ejercicios/ej10/data/inventario_limpio.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventario_limpio" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inventario_limpio" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,16 @@
           <t>categoria</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>precio</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -447,6 +457,12 @@
           <t>ELECTRÓNICA</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>899.99</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -462,6 +478,12 @@
           <t>PERIFÉRICOS</t>
         </is>
       </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -477,6 +499,12 @@
           <t>ELECTRÓNICA</t>
         </is>
       </c>
+      <c r="D4" t="n">
+        <v>249</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -492,6 +520,12 @@
           <t>PERIFÉRICOS</t>
         </is>
       </c>
+      <c r="D5" t="n">
+        <v>64.98999999999999</v>
+      </c>
+      <c r="E5" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -506,6 +540,12 @@
         <is>
           <t>ELECTRÓNICA</t>
         </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>